<commit_message>
Update dates to 2026-02-28 and add price data with color-coded percentage changes
</commit_message>
<xml_diff>
--- a/价格数据初步调整_客户B.xlsx
+++ b/价格数据初步调整_客户B.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F623"/>
+  <dimension ref="A1:F699"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -14114,16 +14114,16 @@
         </is>
       </c>
       <c r="C622" t="n">
-        <v>48.48</v>
+        <v>50.87</v>
       </c>
       <c r="D622" t="n">
-        <v>48.65</v>
+        <v>51.16</v>
       </c>
       <c r="E622" t="n">
-        <v>48.3</v>
+        <v>50.68</v>
       </c>
       <c r="F622" t="n">
-        <v>48.5</v>
+        <v>51</v>
       </c>
     </row>
     <row r="623">
@@ -14136,16 +14136,1688 @@
         </is>
       </c>
       <c r="C623" t="n">
-        <v>60.73</v>
+        <v>63.45</v>
       </c>
       <c r="D623" t="n">
-        <v>60.93</v>
+        <v>64.14</v>
       </c>
       <c r="E623" t="n">
-        <v>60.61</v>
+        <v>63.33</v>
       </c>
       <c r="F623" t="n">
-        <v>60.8</v>
+        <v>64</v>
+      </c>
+    </row>
+    <row r="624">
+      <c r="A624" s="2" t="n">
+        <v>46026</v>
+      </c>
+      <c r="B624" t="inlineStr">
+        <is>
+          <t>牛前八件套</t>
+        </is>
+      </c>
+      <c r="C624" t="n">
+        <v>51.34</v>
+      </c>
+      <c r="D624" t="n">
+        <v>51.5</v>
+      </c>
+      <c r="E624" t="n">
+        <v>51.12</v>
+      </c>
+      <c r="F624" t="n">
+        <v>51.4</v>
+      </c>
+    </row>
+    <row r="625">
+      <c r="A625" s="2" t="n">
+        <v>46026</v>
+      </c>
+      <c r="B625" t="inlineStr">
+        <is>
+          <t>龟排腱</t>
+        </is>
+      </c>
+      <c r="C625" t="n">
+        <v>64.86</v>
+      </c>
+      <c r="D625" t="n">
+        <v>65.06</v>
+      </c>
+      <c r="E625" t="n">
+        <v>64.56</v>
+      </c>
+      <c r="F625" t="n">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="626">
+      <c r="A626" s="2" t="n">
+        <v>46027</v>
+      </c>
+      <c r="B626" t="inlineStr">
+        <is>
+          <t>牛前八件套</t>
+        </is>
+      </c>
+      <c r="C626" t="n">
+        <v>51.49</v>
+      </c>
+      <c r="D626" t="n">
+        <v>51.61</v>
+      </c>
+      <c r="E626" t="n">
+        <v>51.35</v>
+      </c>
+      <c r="F626" t="n">
+        <v>51.5</v>
+      </c>
+    </row>
+    <row r="627">
+      <c r="A627" s="2" t="n">
+        <v>46027</v>
+      </c>
+      <c r="B627" t="inlineStr">
+        <is>
+          <t>龟排腱</t>
+        </is>
+      </c>
+      <c r="C627" t="n">
+        <v>65.48999999999999</v>
+      </c>
+      <c r="D627" t="n">
+        <v>65.58</v>
+      </c>
+      <c r="E627" t="n">
+        <v>64.68000000000001</v>
+      </c>
+      <c r="F627" t="n">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="628">
+      <c r="A628" s="2" t="n">
+        <v>46028</v>
+      </c>
+      <c r="B628" t="inlineStr">
+        <is>
+          <t>牛前八件套</t>
+        </is>
+      </c>
+      <c r="C628" t="n">
+        <v>51.03</v>
+      </c>
+      <c r="D628" t="n">
+        <v>51.23</v>
+      </c>
+      <c r="E628" t="n">
+        <v>50.97</v>
+      </c>
+      <c r="F628" t="n">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="629">
+      <c r="A629" s="2" t="n">
+        <v>46028</v>
+      </c>
+      <c r="B629" t="inlineStr">
+        <is>
+          <t>龟排腱</t>
+        </is>
+      </c>
+      <c r="C629" t="n">
+        <v>65.67</v>
+      </c>
+      <c r="D629" t="n">
+        <v>66.27</v>
+      </c>
+      <c r="E629" t="n">
+        <v>65.48999999999999</v>
+      </c>
+      <c r="F629" t="n">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="630">
+      <c r="A630" s="2" t="n">
+        <v>46029</v>
+      </c>
+      <c r="B630" t="inlineStr">
+        <is>
+          <t>牛前八件套</t>
+        </is>
+      </c>
+      <c r="C630" t="n">
+        <v>51.6</v>
+      </c>
+      <c r="D630" t="n">
+        <v>52.3</v>
+      </c>
+      <c r="E630" t="n">
+        <v>51.55</v>
+      </c>
+      <c r="F630" t="n">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="631">
+      <c r="A631" s="2" t="n">
+        <v>46029</v>
+      </c>
+      <c r="B631" t="inlineStr">
+        <is>
+          <t>龟排腱</t>
+        </is>
+      </c>
+      <c r="C631" t="n">
+        <v>65.66</v>
+      </c>
+      <c r="D631" t="n">
+        <v>66.05</v>
+      </c>
+      <c r="E631" t="n">
+        <v>65.36</v>
+      </c>
+      <c r="F631" t="n">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="632">
+      <c r="A632" s="2" t="n">
+        <v>46030</v>
+      </c>
+      <c r="B632" t="inlineStr">
+        <is>
+          <t>牛前八件套</t>
+        </is>
+      </c>
+      <c r="C632" t="n">
+        <v>51.49</v>
+      </c>
+      <c r="D632" t="n">
+        <v>52.32</v>
+      </c>
+      <c r="E632" t="n">
+        <v>51.3</v>
+      </c>
+      <c r="F632" t="n">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="633">
+      <c r="A633" s="2" t="n">
+        <v>46030</v>
+      </c>
+      <c r="B633" t="inlineStr">
+        <is>
+          <t>龟排腱</t>
+        </is>
+      </c>
+      <c r="C633" t="n">
+        <v>66.63</v>
+      </c>
+      <c r="D633" t="n">
+        <v>67.31999999999999</v>
+      </c>
+      <c r="E633" t="n">
+        <v>66.52</v>
+      </c>
+      <c r="F633" t="n">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="634">
+      <c r="A634" s="2" t="n">
+        <v>46031</v>
+      </c>
+      <c r="B634" t="inlineStr">
+        <is>
+          <t>牛前八件套</t>
+        </is>
+      </c>
+      <c r="C634" t="n">
+        <v>52.24</v>
+      </c>
+      <c r="D634" t="n">
+        <v>52.44</v>
+      </c>
+      <c r="E634" t="n">
+        <v>51.97</v>
+      </c>
+      <c r="F634" t="n">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="635">
+      <c r="A635" s="2" t="n">
+        <v>46031</v>
+      </c>
+      <c r="B635" t="inlineStr">
+        <is>
+          <t>龟排腱</t>
+        </is>
+      </c>
+      <c r="C635" t="n">
+        <v>66.8</v>
+      </c>
+      <c r="D635" t="n">
+        <v>67.36</v>
+      </c>
+      <c r="E635" t="n">
+        <v>66.5</v>
+      </c>
+      <c r="F635" t="n">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="636">
+      <c r="A636" s="2" t="n">
+        <v>46034</v>
+      </c>
+      <c r="B636" t="inlineStr">
+        <is>
+          <t>牛前八件套</t>
+        </is>
+      </c>
+      <c r="C636" t="n">
+        <v>52.85</v>
+      </c>
+      <c r="D636" t="n">
+        <v>53.05</v>
+      </c>
+      <c r="E636" t="n">
+        <v>52.63</v>
+      </c>
+      <c r="F636" t="n">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="637">
+      <c r="A637" s="2" t="n">
+        <v>46034</v>
+      </c>
+      <c r="B637" t="inlineStr">
+        <is>
+          <t>龟排腱</t>
+        </is>
+      </c>
+      <c r="C637" t="n">
+        <v>67.64</v>
+      </c>
+      <c r="D637" t="n">
+        <v>68.40000000000001</v>
+      </c>
+      <c r="E637" t="n">
+        <v>67.42</v>
+      </c>
+      <c r="F637" t="n">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="638">
+      <c r="A638" s="2" t="n">
+        <v>46035</v>
+      </c>
+      <c r="B638" t="inlineStr">
+        <is>
+          <t>牛前八件套</t>
+        </is>
+      </c>
+      <c r="C638" t="n">
+        <v>53.3</v>
+      </c>
+      <c r="D638" t="n">
+        <v>53.53</v>
+      </c>
+      <c r="E638" t="n">
+        <v>53.28</v>
+      </c>
+      <c r="F638" t="n">
+        <v>53.4</v>
+      </c>
+    </row>
+    <row r="639">
+      <c r="A639" s="2" t="n">
+        <v>46035</v>
+      </c>
+      <c r="B639" t="inlineStr">
+        <is>
+          <t>龟排腱</t>
+        </is>
+      </c>
+      <c r="C639" t="n">
+        <v>68.97</v>
+      </c>
+      <c r="D639" t="n">
+        <v>69.08</v>
+      </c>
+      <c r="E639" t="n">
+        <v>68.66</v>
+      </c>
+      <c r="F639" t="n">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="640">
+      <c r="A640" s="2" t="n">
+        <v>46036</v>
+      </c>
+      <c r="B640" t="inlineStr">
+        <is>
+          <t>牛前八件套</t>
+        </is>
+      </c>
+      <c r="C640" t="n">
+        <v>53.58</v>
+      </c>
+      <c r="D640" t="n">
+        <v>53.73</v>
+      </c>
+      <c r="E640" t="n">
+        <v>53.38</v>
+      </c>
+      <c r="F640" t="n">
+        <v>53.6</v>
+      </c>
+    </row>
+    <row r="641">
+      <c r="A641" s="2" t="n">
+        <v>46036</v>
+      </c>
+      <c r="B641" t="inlineStr">
+        <is>
+          <t>龟排腱</t>
+        </is>
+      </c>
+      <c r="C641" t="n">
+        <v>69.75</v>
+      </c>
+      <c r="D641" t="n">
+        <v>70</v>
+      </c>
+      <c r="E641" t="n">
+        <v>69.72</v>
+      </c>
+      <c r="F641" t="n">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="642">
+      <c r="A642" s="2" t="n">
+        <v>46037</v>
+      </c>
+      <c r="B642" t="inlineStr">
+        <is>
+          <t>牛前八件套</t>
+        </is>
+      </c>
+      <c r="C642" t="n">
+        <v>54.27</v>
+      </c>
+      <c r="D642" t="n">
+        <v>54.86</v>
+      </c>
+      <c r="E642" t="n">
+        <v>54.14</v>
+      </c>
+      <c r="F642" t="n">
+        <v>54.5</v>
+      </c>
+    </row>
+    <row r="643">
+      <c r="A643" s="2" t="n">
+        <v>46037</v>
+      </c>
+      <c r="B643" t="inlineStr">
+        <is>
+          <t>龟排腱</t>
+        </is>
+      </c>
+      <c r="C643" t="n">
+        <v>70.73</v>
+      </c>
+      <c r="D643" t="n">
+        <v>71</v>
+      </c>
+      <c r="E643" t="n">
+        <v>70.67</v>
+      </c>
+      <c r="F643" t="n">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="644">
+      <c r="A644" s="2" t="n">
+        <v>46038</v>
+      </c>
+      <c r="B644" t="inlineStr">
+        <is>
+          <t>牛前八件套</t>
+        </is>
+      </c>
+      <c r="C644" t="n">
+        <v>54.7</v>
+      </c>
+      <c r="D644" t="n">
+        <v>55.03</v>
+      </c>
+      <c r="E644" t="n">
+        <v>54.51</v>
+      </c>
+      <c r="F644" t="n">
+        <v>54.7</v>
+      </c>
+    </row>
+    <row r="645">
+      <c r="A645" s="2" t="n">
+        <v>46038</v>
+      </c>
+      <c r="B645" t="inlineStr">
+        <is>
+          <t>龟排腱</t>
+        </is>
+      </c>
+      <c r="C645" t="n">
+        <v>70.75</v>
+      </c>
+      <c r="D645" t="n">
+        <v>71.40000000000001</v>
+      </c>
+      <c r="E645" t="n">
+        <v>70.52</v>
+      </c>
+      <c r="F645" t="n">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="646">
+      <c r="A646" s="2" t="n">
+        <v>46041</v>
+      </c>
+      <c r="B646" t="inlineStr">
+        <is>
+          <t>牛前八件套</t>
+        </is>
+      </c>
+      <c r="C646" t="n">
+        <v>54.95</v>
+      </c>
+      <c r="D646" t="n">
+        <v>55.16</v>
+      </c>
+      <c r="E646" t="n">
+        <v>54.67</v>
+      </c>
+      <c r="F646" t="n">
+        <v>54.7</v>
+      </c>
+    </row>
+    <row r="647">
+      <c r="A647" s="2" t="n">
+        <v>46041</v>
+      </c>
+      <c r="B647" t="inlineStr">
+        <is>
+          <t>龟排腱</t>
+        </is>
+      </c>
+      <c r="C647" t="n">
+        <v>70.93000000000001</v>
+      </c>
+      <c r="D647" t="n">
+        <v>71.17</v>
+      </c>
+      <c r="E647" t="n">
+        <v>70.59999999999999</v>
+      </c>
+      <c r="F647" t="n">
+        <v>70.90000000000001</v>
+      </c>
+    </row>
+    <row r="648">
+      <c r="A648" s="2" t="n">
+        <v>46042</v>
+      </c>
+      <c r="B648" t="inlineStr">
+        <is>
+          <t>牛前八件套</t>
+        </is>
+      </c>
+      <c r="C648" t="n">
+        <v>54.55</v>
+      </c>
+      <c r="D648" t="n">
+        <v>54.75</v>
+      </c>
+      <c r="E648" t="n">
+        <v>54.31</v>
+      </c>
+      <c r="F648" t="n">
+        <v>54.7</v>
+      </c>
+    </row>
+    <row r="649">
+      <c r="A649" s="2" t="n">
+        <v>46042</v>
+      </c>
+      <c r="B649" t="inlineStr">
+        <is>
+          <t>龟排腱</t>
+        </is>
+      </c>
+      <c r="C649" t="n">
+        <v>70.8</v>
+      </c>
+      <c r="D649" t="n">
+        <v>70.93000000000001</v>
+      </c>
+      <c r="E649" t="n">
+        <v>70.66</v>
+      </c>
+      <c r="F649" t="n">
+        <v>70.8</v>
+      </c>
+    </row>
+    <row r="650">
+      <c r="A650" s="2" t="n">
+        <v>46043</v>
+      </c>
+      <c r="B650" t="inlineStr">
+        <is>
+          <t>牛前八件套</t>
+        </is>
+      </c>
+      <c r="C650" t="n">
+        <v>54.83</v>
+      </c>
+      <c r="D650" t="n">
+        <v>54.93</v>
+      </c>
+      <c r="E650" t="n">
+        <v>54.67</v>
+      </c>
+      <c r="F650" t="n">
+        <v>54.7</v>
+      </c>
+    </row>
+    <row r="651">
+      <c r="A651" s="2" t="n">
+        <v>46043</v>
+      </c>
+      <c r="B651" t="inlineStr">
+        <is>
+          <t>龟排腱</t>
+        </is>
+      </c>
+      <c r="C651" t="n">
+        <v>70.70999999999999</v>
+      </c>
+      <c r="D651" t="n">
+        <v>71.05</v>
+      </c>
+      <c r="E651" t="n">
+        <v>70.48999999999999</v>
+      </c>
+      <c r="F651" t="n">
+        <v>70.7</v>
+      </c>
+    </row>
+    <row r="652">
+      <c r="A652" s="2" t="n">
+        <v>46044</v>
+      </c>
+      <c r="B652" t="inlineStr">
+        <is>
+          <t>牛前八件套</t>
+        </is>
+      </c>
+      <c r="C652" t="n">
+        <v>54.49</v>
+      </c>
+      <c r="D652" t="n">
+        <v>54.83</v>
+      </c>
+      <c r="E652" t="n">
+        <v>54.29</v>
+      </c>
+      <c r="F652" t="n">
+        <v>54.7</v>
+      </c>
+    </row>
+    <row r="653">
+      <c r="A653" s="2" t="n">
+        <v>46044</v>
+      </c>
+      <c r="B653" t="inlineStr">
+        <is>
+          <t>龟排腱</t>
+        </is>
+      </c>
+      <c r="C653" t="n">
+        <v>71.25</v>
+      </c>
+      <c r="D653" t="n">
+        <v>71.48</v>
+      </c>
+      <c r="E653" t="n">
+        <v>70.28</v>
+      </c>
+      <c r="F653" t="n">
+        <v>70.7</v>
+      </c>
+    </row>
+    <row r="654">
+      <c r="A654" s="2" t="n">
+        <v>46045</v>
+      </c>
+      <c r="B654" t="inlineStr">
+        <is>
+          <t>牛前八件套</t>
+        </is>
+      </c>
+      <c r="C654" t="n">
+        <v>54.55</v>
+      </c>
+      <c r="D654" t="n">
+        <v>54.79</v>
+      </c>
+      <c r="E654" t="n">
+        <v>54.31</v>
+      </c>
+      <c r="F654" t="n">
+        <v>54.5</v>
+      </c>
+    </row>
+    <row r="655">
+      <c r="A655" s="2" t="n">
+        <v>46045</v>
+      </c>
+      <c r="B655" t="inlineStr">
+        <is>
+          <t>龟排腱</t>
+        </is>
+      </c>
+      <c r="C655" t="n">
+        <v>70.62</v>
+      </c>
+      <c r="D655" t="n">
+        <v>70.81999999999999</v>
+      </c>
+      <c r="E655" t="n">
+        <v>70.34</v>
+      </c>
+      <c r="F655" t="n">
+        <v>70.59999999999999</v>
+      </c>
+    </row>
+    <row r="656">
+      <c r="A656" s="2" t="n">
+        <v>46048</v>
+      </c>
+      <c r="B656" t="inlineStr">
+        <is>
+          <t>牛前八件套</t>
+        </is>
+      </c>
+      <c r="C656" t="n">
+        <v>54.09</v>
+      </c>
+      <c r="D656" t="n">
+        <v>54.79</v>
+      </c>
+      <c r="E656" t="n">
+        <v>53.88</v>
+      </c>
+      <c r="F656" t="n">
+        <v>54.5</v>
+      </c>
+    </row>
+    <row r="657">
+      <c r="A657" s="2" t="n">
+        <v>46048</v>
+      </c>
+      <c r="B657" t="inlineStr">
+        <is>
+          <t>龟排腱</t>
+        </is>
+      </c>
+      <c r="C657" t="n">
+        <v>70.17</v>
+      </c>
+      <c r="D657" t="n">
+        <v>70.98</v>
+      </c>
+      <c r="E657" t="n">
+        <v>70.06999999999999</v>
+      </c>
+      <c r="F657" t="n">
+        <v>70.59999999999999</v>
+      </c>
+    </row>
+    <row r="658">
+      <c r="A658" s="2" t="n">
+        <v>46049</v>
+      </c>
+      <c r="B658" t="inlineStr">
+        <is>
+          <t>牛前八件套</t>
+        </is>
+      </c>
+      <c r="C658" t="n">
+        <v>54.19</v>
+      </c>
+      <c r="D658" t="n">
+        <v>54.4</v>
+      </c>
+      <c r="E658" t="n">
+        <v>53.9</v>
+      </c>
+      <c r="F658" t="n">
+        <v>54.1</v>
+      </c>
+    </row>
+    <row r="659">
+      <c r="A659" s="2" t="n">
+        <v>46049</v>
+      </c>
+      <c r="B659" t="inlineStr">
+        <is>
+          <t>龟排腱</t>
+        </is>
+      </c>
+      <c r="C659" t="n">
+        <v>70.5</v>
+      </c>
+      <c r="D659" t="n">
+        <v>70.73</v>
+      </c>
+      <c r="E659" t="n">
+        <v>70.41</v>
+      </c>
+      <c r="F659" t="n">
+        <v>70.5</v>
+      </c>
+    </row>
+    <row r="660">
+      <c r="A660" s="2" t="n">
+        <v>46050</v>
+      </c>
+      <c r="B660" t="inlineStr">
+        <is>
+          <t>牛前八件套</t>
+        </is>
+      </c>
+      <c r="C660" t="n">
+        <v>54.18</v>
+      </c>
+      <c r="D660" t="n">
+        <v>54.37</v>
+      </c>
+      <c r="E660" t="n">
+        <v>54.17</v>
+      </c>
+      <c r="F660" t="n">
+        <v>54.2</v>
+      </c>
+    </row>
+    <row r="661">
+      <c r="A661" s="2" t="n">
+        <v>46050</v>
+      </c>
+      <c r="B661" t="inlineStr">
+        <is>
+          <t>龟排腱</t>
+        </is>
+      </c>
+      <c r="C661" t="n">
+        <v>71.12</v>
+      </c>
+      <c r="D661" t="n">
+        <v>71.45999999999999</v>
+      </c>
+      <c r="E661" t="n">
+        <v>70.02</v>
+      </c>
+      <c r="F661" t="n">
+        <v>70.5</v>
+      </c>
+    </row>
+    <row r="662">
+      <c r="A662" s="2" t="n">
+        <v>46051</v>
+      </c>
+      <c r="B662" t="inlineStr">
+        <is>
+          <t>牛前八件套</t>
+        </is>
+      </c>
+      <c r="C662" t="n">
+        <v>53.77</v>
+      </c>
+      <c r="D662" t="n">
+        <v>54.21</v>
+      </c>
+      <c r="E662" t="n">
+        <v>53.6</v>
+      </c>
+      <c r="F662" t="n">
+        <v>54.2</v>
+      </c>
+    </row>
+    <row r="663">
+      <c r="A663" s="2" t="n">
+        <v>46051</v>
+      </c>
+      <c r="B663" t="inlineStr">
+        <is>
+          <t>龟排腱</t>
+        </is>
+      </c>
+      <c r="C663" t="n">
+        <v>70.31999999999999</v>
+      </c>
+      <c r="D663" t="n">
+        <v>70.51000000000001</v>
+      </c>
+      <c r="E663" t="n">
+        <v>69.98999999999999</v>
+      </c>
+      <c r="F663" t="n">
+        <v>70.5</v>
+      </c>
+    </row>
+    <row r="664">
+      <c r="A664" s="2" t="n">
+        <v>46052</v>
+      </c>
+      <c r="B664" t="inlineStr">
+        <is>
+          <t>牛前八件套</t>
+        </is>
+      </c>
+      <c r="C664" t="n">
+        <v>54</v>
+      </c>
+      <c r="D664" t="n">
+        <v>54.41</v>
+      </c>
+      <c r="E664" t="n">
+        <v>53.75</v>
+      </c>
+      <c r="F664" t="n">
+        <v>54.2</v>
+      </c>
+    </row>
+    <row r="665">
+      <c r="A665" s="2" t="n">
+        <v>46052</v>
+      </c>
+      <c r="B665" t="inlineStr">
+        <is>
+          <t>龟排腱</t>
+        </is>
+      </c>
+      <c r="C665" t="n">
+        <v>70.40000000000001</v>
+      </c>
+      <c r="D665" t="n">
+        <v>71.01000000000001</v>
+      </c>
+      <c r="E665" t="n">
+        <v>70.06</v>
+      </c>
+      <c r="F665" t="n">
+        <v>70.5</v>
+      </c>
+    </row>
+    <row r="666">
+      <c r="A666" s="2" t="n">
+        <v>46053</v>
+      </c>
+      <c r="B666" t="inlineStr">
+        <is>
+          <t>牛前八件套</t>
+        </is>
+      </c>
+      <c r="C666" t="n">
+        <v>53.93</v>
+      </c>
+      <c r="D666" t="n">
+        <v>54.37</v>
+      </c>
+      <c r="E666" t="n">
+        <v>53.72</v>
+      </c>
+      <c r="F666" t="n">
+        <v>54.2</v>
+      </c>
+    </row>
+    <row r="667">
+      <c r="A667" s="2" t="n">
+        <v>46053</v>
+      </c>
+      <c r="B667" t="inlineStr">
+        <is>
+          <t>龟排腱</t>
+        </is>
+      </c>
+      <c r="C667" t="n">
+        <v>71</v>
+      </c>
+      <c r="D667" t="n">
+        <v>71.09999999999999</v>
+      </c>
+      <c r="E667" t="n">
+        <v>70.3</v>
+      </c>
+      <c r="F667" t="n">
+        <v>70.5</v>
+      </c>
+    </row>
+    <row r="668">
+      <c r="A668" s="2" t="n">
+        <v>46055</v>
+      </c>
+      <c r="B668" t="inlineStr">
+        <is>
+          <t>牛前八件套</t>
+        </is>
+      </c>
+      <c r="C668" t="n">
+        <v>53.8</v>
+      </c>
+      <c r="D668" t="n">
+        <v>53.92</v>
+      </c>
+      <c r="E668" t="n">
+        <v>53.69</v>
+      </c>
+      <c r="F668" t="n">
+        <v>53.7</v>
+      </c>
+    </row>
+    <row r="669">
+      <c r="A669" s="2" t="n">
+        <v>46055</v>
+      </c>
+      <c r="B669" t="inlineStr">
+        <is>
+          <t>龟排腱</t>
+        </is>
+      </c>
+      <c r="C669" t="n">
+        <v>70.2</v>
+      </c>
+      <c r="D669" t="n">
+        <v>70.81</v>
+      </c>
+      <c r="E669" t="n">
+        <v>70.19</v>
+      </c>
+      <c r="F669" t="n">
+        <v>70.5</v>
+      </c>
+    </row>
+    <row r="670">
+      <c r="A670" s="2" t="n">
+        <v>46056</v>
+      </c>
+      <c r="B670" t="inlineStr">
+        <is>
+          <t>牛前八件套</t>
+        </is>
+      </c>
+      <c r="C670" t="n">
+        <v>53.28</v>
+      </c>
+      <c r="D670" t="n">
+        <v>53.71</v>
+      </c>
+      <c r="E670" t="n">
+        <v>53.11</v>
+      </c>
+      <c r="F670" t="n">
+        <v>53.7</v>
+      </c>
+    </row>
+    <row r="671">
+      <c r="A671" s="2" t="n">
+        <v>46056</v>
+      </c>
+      <c r="B671" t="inlineStr">
+        <is>
+          <t>龟排腱</t>
+        </is>
+      </c>
+      <c r="C671" t="n">
+        <v>69.84999999999999</v>
+      </c>
+      <c r="D671" t="n">
+        <v>70.93000000000001</v>
+      </c>
+      <c r="E671" t="n">
+        <v>69.72</v>
+      </c>
+      <c r="F671" t="n">
+        <v>70.5</v>
+      </c>
+    </row>
+    <row r="672">
+      <c r="A672" s="2" t="n">
+        <v>46057</v>
+      </c>
+      <c r="B672" t="inlineStr">
+        <is>
+          <t>牛前八件套</t>
+        </is>
+      </c>
+      <c r="C672" t="n">
+        <v>53.96</v>
+      </c>
+      <c r="D672" t="n">
+        <v>54.21</v>
+      </c>
+      <c r="E672" t="n">
+        <v>53.72</v>
+      </c>
+      <c r="F672" t="n">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="673">
+      <c r="A673" s="2" t="n">
+        <v>46057</v>
+      </c>
+      <c r="B673" t="inlineStr">
+        <is>
+          <t>龟排腱</t>
+        </is>
+      </c>
+      <c r="C673" t="n">
+        <v>70.59</v>
+      </c>
+      <c r="D673" t="n">
+        <v>70.88</v>
+      </c>
+      <c r="E673" t="n">
+        <v>70.31999999999999</v>
+      </c>
+      <c r="F673" t="n">
+        <v>70.59999999999999</v>
+      </c>
+    </row>
+    <row r="674">
+      <c r="A674" s="2" t="n">
+        <v>46058</v>
+      </c>
+      <c r="B674" t="inlineStr">
+        <is>
+          <t>牛前八件套</t>
+        </is>
+      </c>
+      <c r="C674" t="n">
+        <v>53.73</v>
+      </c>
+      <c r="D674" t="n">
+        <v>54.17</v>
+      </c>
+      <c r="E674" t="n">
+        <v>53.53</v>
+      </c>
+      <c r="F674" t="n">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="675">
+      <c r="A675" s="2" t="n">
+        <v>46058</v>
+      </c>
+      <c r="B675" t="inlineStr">
+        <is>
+          <t>龟排腱</t>
+        </is>
+      </c>
+      <c r="C675" t="n">
+        <v>70.69</v>
+      </c>
+      <c r="D675" t="n">
+        <v>71.03</v>
+      </c>
+      <c r="E675" t="n">
+        <v>70.66</v>
+      </c>
+      <c r="F675" t="n">
+        <v>70.7</v>
+      </c>
+    </row>
+    <row r="676">
+      <c r="A676" s="2" t="n">
+        <v>46059</v>
+      </c>
+      <c r="B676" t="inlineStr">
+        <is>
+          <t>牛前八件套</t>
+        </is>
+      </c>
+      <c r="C676" t="n">
+        <v>53.71</v>
+      </c>
+      <c r="D676" t="n">
+        <v>54.03</v>
+      </c>
+      <c r="E676" t="n">
+        <v>53.63</v>
+      </c>
+      <c r="F676" t="n">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="677">
+      <c r="A677" s="2" t="n">
+        <v>46059</v>
+      </c>
+      <c r="B677" t="inlineStr">
+        <is>
+          <t>龟排腱</t>
+        </is>
+      </c>
+      <c r="C677" t="n">
+        <v>70.06999999999999</v>
+      </c>
+      <c r="D677" t="n">
+        <v>70.98</v>
+      </c>
+      <c r="E677" t="n">
+        <v>69.88</v>
+      </c>
+      <c r="F677" t="n">
+        <v>70.7</v>
+      </c>
+    </row>
+    <row r="678">
+      <c r="A678" s="2" t="n">
+        <v>46062</v>
+      </c>
+      <c r="B678" t="inlineStr">
+        <is>
+          <t>牛前八件套</t>
+        </is>
+      </c>
+      <c r="C678" t="n">
+        <v>53.63</v>
+      </c>
+      <c r="D678" t="n">
+        <v>54.38</v>
+      </c>
+      <c r="E678" t="n">
+        <v>53.42</v>
+      </c>
+      <c r="F678" t="n">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="679">
+      <c r="A679" s="2" t="n">
+        <v>46062</v>
+      </c>
+      <c r="B679" t="inlineStr">
+        <is>
+          <t>龟排腱</t>
+        </is>
+      </c>
+      <c r="C679" t="n">
+        <v>70.77</v>
+      </c>
+      <c r="D679" t="n">
+        <v>71.19</v>
+      </c>
+      <c r="E679" t="n">
+        <v>70.43000000000001</v>
+      </c>
+      <c r="F679" t="n">
+        <v>70.8</v>
+      </c>
+    </row>
+    <row r="680">
+      <c r="A680" s="2" t="n">
+        <v>46063</v>
+      </c>
+      <c r="B680" t="inlineStr">
+        <is>
+          <t>牛前八件套</t>
+        </is>
+      </c>
+      <c r="C680" t="n">
+        <v>54.14</v>
+      </c>
+      <c r="D680" t="n">
+        <v>54.38</v>
+      </c>
+      <c r="E680" t="n">
+        <v>53.67</v>
+      </c>
+      <c r="F680" t="n">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="681">
+      <c r="A681" s="2" t="n">
+        <v>46063</v>
+      </c>
+      <c r="B681" t="inlineStr">
+        <is>
+          <t>龟排腱</t>
+        </is>
+      </c>
+      <c r="C681" t="n">
+        <v>70.81999999999999</v>
+      </c>
+      <c r="D681" t="n">
+        <v>70.94</v>
+      </c>
+      <c r="E681" t="n">
+        <v>70.38</v>
+      </c>
+      <c r="F681" t="n">
+        <v>70.8</v>
+      </c>
+    </row>
+    <row r="682">
+      <c r="A682" s="2" t="n">
+        <v>46064</v>
+      </c>
+      <c r="B682" t="inlineStr">
+        <is>
+          <t>牛前八件套</t>
+        </is>
+      </c>
+      <c r="C682" t="n">
+        <v>54.46</v>
+      </c>
+      <c r="D682" t="n">
+        <v>54.86</v>
+      </c>
+      <c r="E682" t="n">
+        <v>54.32</v>
+      </c>
+      <c r="F682" t="n">
+        <v>54.5</v>
+      </c>
+    </row>
+    <row r="683">
+      <c r="A683" s="2" t="n">
+        <v>46064</v>
+      </c>
+      <c r="B683" t="inlineStr">
+        <is>
+          <t>龟排腱</t>
+        </is>
+      </c>
+      <c r="C683" t="n">
+        <v>70.48</v>
+      </c>
+      <c r="D683" t="n">
+        <v>71.03</v>
+      </c>
+      <c r="E683" t="n">
+        <v>70.45</v>
+      </c>
+      <c r="F683" t="n">
+        <v>70.8</v>
+      </c>
+    </row>
+    <row r="684">
+      <c r="A684" s="2" t="n">
+        <v>46065</v>
+      </c>
+      <c r="B684" t="inlineStr">
+        <is>
+          <t>牛前八件套</t>
+        </is>
+      </c>
+      <c r="C684" t="n">
+        <v>54.84</v>
+      </c>
+      <c r="D684" t="n">
+        <v>55.08</v>
+      </c>
+      <c r="E684" t="n">
+        <v>54.37</v>
+      </c>
+      <c r="F684" t="n">
+        <v>54.5</v>
+      </c>
+    </row>
+    <row r="685">
+      <c r="A685" s="2" t="n">
+        <v>46065</v>
+      </c>
+      <c r="B685" t="inlineStr">
+        <is>
+          <t>龟排腱</t>
+        </is>
+      </c>
+      <c r="C685" t="n">
+        <v>70.13</v>
+      </c>
+      <c r="D685" t="n">
+        <v>71.31</v>
+      </c>
+      <c r="E685" t="n">
+        <v>69.83</v>
+      </c>
+      <c r="F685" t="n">
+        <v>70.8</v>
+      </c>
+    </row>
+    <row r="686">
+      <c r="A686" s="2" t="n">
+        <v>46066</v>
+      </c>
+      <c r="B686" t="inlineStr">
+        <is>
+          <t>牛前八件套</t>
+        </is>
+      </c>
+      <c r="C686" t="n">
+        <v>54.07</v>
+      </c>
+      <c r="D686" t="n">
+        <v>54.59</v>
+      </c>
+      <c r="E686" t="n">
+        <v>53.96</v>
+      </c>
+      <c r="F686" t="n">
+        <v>54.5</v>
+      </c>
+    </row>
+    <row r="687">
+      <c r="A687" s="2" t="n">
+        <v>46066</v>
+      </c>
+      <c r="B687" t="inlineStr">
+        <is>
+          <t>龟排腱</t>
+        </is>
+      </c>
+      <c r="C687" t="n">
+        <v>71.08</v>
+      </c>
+      <c r="D687" t="n">
+        <v>71.22</v>
+      </c>
+      <c r="E687" t="n">
+        <v>70.70999999999999</v>
+      </c>
+      <c r="F687" t="n">
+        <v>70.8</v>
+      </c>
+    </row>
+    <row r="688">
+      <c r="A688" s="2" t="n">
+        <v>46069</v>
+      </c>
+      <c r="B688" t="inlineStr">
+        <is>
+          <t>牛前八件套</t>
+        </is>
+      </c>
+      <c r="C688" t="n">
+        <v>54.85</v>
+      </c>
+      <c r="D688" t="n">
+        <v>55.08</v>
+      </c>
+      <c r="E688" t="n">
+        <v>54.5</v>
+      </c>
+      <c r="F688" t="n">
+        <v>54.5</v>
+      </c>
+    </row>
+    <row r="689">
+      <c r="A689" s="2" t="n">
+        <v>46069</v>
+      </c>
+      <c r="B689" t="inlineStr">
+        <is>
+          <t>龟排腱</t>
+        </is>
+      </c>
+      <c r="C689" t="n">
+        <v>70.31</v>
+      </c>
+      <c r="D689" t="n">
+        <v>70.93000000000001</v>
+      </c>
+      <c r="E689" t="n">
+        <v>70.12</v>
+      </c>
+      <c r="F689" t="n">
+        <v>70.8</v>
+      </c>
+    </row>
+    <row r="690">
+      <c r="A690" s="2" t="n">
+        <v>46077</v>
+      </c>
+      <c r="B690" t="inlineStr">
+        <is>
+          <t>牛前八件套</t>
+        </is>
+      </c>
+      <c r="C690" t="n">
+        <v>55.13</v>
+      </c>
+      <c r="D690" t="n">
+        <v>55.47</v>
+      </c>
+      <c r="E690" t="n">
+        <v>55.07</v>
+      </c>
+      <c r="F690" t="n">
+        <v>55.3</v>
+      </c>
+    </row>
+    <row r="691">
+      <c r="A691" s="2" t="n">
+        <v>46077</v>
+      </c>
+      <c r="B691" t="inlineStr">
+        <is>
+          <t>龟排腱</t>
+        </is>
+      </c>
+      <c r="C691" t="n">
+        <v>71.09999999999999</v>
+      </c>
+      <c r="D691" t="n">
+        <v>71.34</v>
+      </c>
+      <c r="E691" t="n">
+        <v>70.65000000000001</v>
+      </c>
+      <c r="F691" t="n">
+        <v>70.8</v>
+      </c>
+    </row>
+    <row r="692">
+      <c r="A692" s="2" t="n">
+        <v>46078</v>
+      </c>
+      <c r="B692" t="inlineStr">
+        <is>
+          <t>牛前八件套</t>
+        </is>
+      </c>
+      <c r="C692" t="n">
+        <v>54.88</v>
+      </c>
+      <c r="D692" t="n">
+        <v>55.44</v>
+      </c>
+      <c r="E692" t="n">
+        <v>54.62</v>
+      </c>
+      <c r="F692" t="n">
+        <v>55.3</v>
+      </c>
+    </row>
+    <row r="693">
+      <c r="A693" s="2" t="n">
+        <v>46078</v>
+      </c>
+      <c r="B693" t="inlineStr">
+        <is>
+          <t>龟排腱</t>
+        </is>
+      </c>
+      <c r="C693" t="n">
+        <v>71.44</v>
+      </c>
+      <c r="D693" t="n">
+        <v>71.70999999999999</v>
+      </c>
+      <c r="E693" t="n">
+        <v>70.51000000000001</v>
+      </c>
+      <c r="F693" t="n">
+        <v>70.8</v>
+      </c>
+    </row>
+    <row r="694">
+      <c r="A694" s="2" t="n">
+        <v>46079</v>
+      </c>
+      <c r="B694" t="inlineStr">
+        <is>
+          <t>牛前八件套</t>
+        </is>
+      </c>
+      <c r="C694" t="n">
+        <v>55.47</v>
+      </c>
+      <c r="D694" t="n">
+        <v>55.72</v>
+      </c>
+      <c r="E694" t="n">
+        <v>55.28</v>
+      </c>
+      <c r="F694" t="n">
+        <v>55.5</v>
+      </c>
+    </row>
+    <row r="695">
+      <c r="A695" s="2" t="n">
+        <v>46079</v>
+      </c>
+      <c r="B695" t="inlineStr">
+        <is>
+          <t>龟排腱</t>
+        </is>
+      </c>
+      <c r="C695" t="n">
+        <v>70.95999999999999</v>
+      </c>
+      <c r="D695" t="n">
+        <v>71.11</v>
+      </c>
+      <c r="E695" t="n">
+        <v>70.67</v>
+      </c>
+      <c r="F695" t="n">
+        <v>70.8</v>
+      </c>
+    </row>
+    <row r="696">
+      <c r="A696" s="2" t="n">
+        <v>46080</v>
+      </c>
+      <c r="B696" t="inlineStr">
+        <is>
+          <t>牛前八件套</t>
+        </is>
+      </c>
+      <c r="C696" t="n">
+        <v>55.67</v>
+      </c>
+      <c r="D696" t="n">
+        <v>56.11</v>
+      </c>
+      <c r="E696" t="n">
+        <v>55.4</v>
+      </c>
+      <c r="F696" t="n">
+        <v>55.7</v>
+      </c>
+    </row>
+    <row r="697">
+      <c r="A697" s="2" t="n">
+        <v>46080</v>
+      </c>
+      <c r="B697" t="inlineStr">
+        <is>
+          <t>龟排腱</t>
+        </is>
+      </c>
+      <c r="C697" t="n">
+        <v>70.59999999999999</v>
+      </c>
+      <c r="D697" t="n">
+        <v>71.2</v>
+      </c>
+      <c r="E697" t="n">
+        <v>70.59</v>
+      </c>
+      <c r="F697" t="n">
+        <v>70.8</v>
+      </c>
+    </row>
+    <row r="698">
+      <c r="A698" s="2" t="n">
+        <v>46081</v>
+      </c>
+      <c r="B698" t="inlineStr">
+        <is>
+          <t>牛前八件套</t>
+        </is>
+      </c>
+      <c r="C698" t="n">
+        <v>55.97</v>
+      </c>
+      <c r="D698" t="n">
+        <v>56.21</v>
+      </c>
+      <c r="E698" t="n">
+        <v>55.89</v>
+      </c>
+      <c r="F698" t="n">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="699">
+      <c r="A699" s="2" t="n">
+        <v>46081</v>
+      </c>
+      <c r="B699" t="inlineStr">
+        <is>
+          <t>龟排腱</t>
+        </is>
+      </c>
+      <c r="C699" t="n">
+        <v>70.26000000000001</v>
+      </c>
+      <c r="D699" t="n">
+        <v>70.81999999999999</v>
+      </c>
+      <c r="E699" t="n">
+        <v>70.23999999999999</v>
+      </c>
+      <c r="F699" t="n">
+        <v>70.8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update HTML reports to 2026-04-30 with new price data
</commit_message>
<xml_diff>
--- a/价格数据初步调整_客户B.xlsx
+++ b/价格数据初步调整_客户B.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F699"/>
+  <dimension ref="A1:F789"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -15820,6 +15820,1986 @@
         <v>70.8</v>
       </c>
     </row>
+    <row r="700">
+      <c r="A700" s="2" t="n">
+        <v>46083</v>
+      </c>
+      <c r="B700" t="inlineStr">
+        <is>
+          <t>牛前八件套</t>
+        </is>
+      </c>
+      <c r="C700" t="n">
+        <v>56.66</v>
+      </c>
+      <c r="D700" t="n">
+        <v>57.04</v>
+      </c>
+      <c r="E700" t="n">
+        <v>56.64</v>
+      </c>
+      <c r="F700" t="n">
+        <v>56.7</v>
+      </c>
+    </row>
+    <row r="701">
+      <c r="A701" s="2" t="n">
+        <v>46083</v>
+      </c>
+      <c r="B701" t="inlineStr">
+        <is>
+          <t>龟排腱</t>
+        </is>
+      </c>
+      <c r="C701" t="n">
+        <v>71.34999999999999</v>
+      </c>
+      <c r="D701" t="n">
+        <v>71.63</v>
+      </c>
+      <c r="E701" t="n">
+        <v>70.45999999999999</v>
+      </c>
+      <c r="F701" t="n">
+        <v>70.8</v>
+      </c>
+    </row>
+    <row r="702">
+      <c r="A702" s="2" t="n">
+        <v>46084</v>
+      </c>
+      <c r="B702" t="inlineStr">
+        <is>
+          <t>牛前八件套</t>
+        </is>
+      </c>
+      <c r="C702" t="n">
+        <v>56.82</v>
+      </c>
+      <c r="D702" t="n">
+        <v>57.23</v>
+      </c>
+      <c r="E702" t="n">
+        <v>56.76</v>
+      </c>
+      <c r="F702" t="n">
+        <v>56.9</v>
+      </c>
+    </row>
+    <row r="703">
+      <c r="A703" s="2" t="n">
+        <v>46084</v>
+      </c>
+      <c r="B703" t="inlineStr">
+        <is>
+          <t>龟排腱</t>
+        </is>
+      </c>
+      <c r="C703" t="n">
+        <v>70.20999999999999</v>
+      </c>
+      <c r="D703" t="n">
+        <v>70.89</v>
+      </c>
+      <c r="E703" t="n">
+        <v>69.90000000000001</v>
+      </c>
+      <c r="F703" t="n">
+        <v>70.8</v>
+      </c>
+    </row>
+    <row r="704">
+      <c r="A704" s="2" t="n">
+        <v>46085</v>
+      </c>
+      <c r="B704" t="inlineStr">
+        <is>
+          <t>牛前八件套</t>
+        </is>
+      </c>
+      <c r="C704" t="n">
+        <v>57</v>
+      </c>
+      <c r="D704" t="n">
+        <v>57.35</v>
+      </c>
+      <c r="E704" t="n">
+        <v>56.8</v>
+      </c>
+      <c r="F704" t="n">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="705">
+      <c r="A705" s="2" t="n">
+        <v>46085</v>
+      </c>
+      <c r="B705" t="inlineStr">
+        <is>
+          <t>龟排腱</t>
+        </is>
+      </c>
+      <c r="C705" t="n">
+        <v>70.95</v>
+      </c>
+      <c r="D705" t="n">
+        <v>70.95</v>
+      </c>
+      <c r="E705" t="n">
+        <v>70.75</v>
+      </c>
+      <c r="F705" t="n">
+        <v>70.8</v>
+      </c>
+    </row>
+    <row r="706">
+      <c r="A706" s="2" t="n">
+        <v>46086</v>
+      </c>
+      <c r="B706" t="inlineStr">
+        <is>
+          <t>牛前八件套</t>
+        </is>
+      </c>
+      <c r="C706" t="n">
+        <v>57.14</v>
+      </c>
+      <c r="D706" t="n">
+        <v>57.53</v>
+      </c>
+      <c r="E706" t="n">
+        <v>57.12</v>
+      </c>
+      <c r="F706" t="n">
+        <v>57.2</v>
+      </c>
+    </row>
+    <row r="707">
+      <c r="A707" s="2" t="n">
+        <v>46086</v>
+      </c>
+      <c r="B707" t="inlineStr">
+        <is>
+          <t>龟排腱</t>
+        </is>
+      </c>
+      <c r="C707" t="n">
+        <v>71.17</v>
+      </c>
+      <c r="D707" t="n">
+        <v>71.3</v>
+      </c>
+      <c r="E707" t="n">
+        <v>71.11</v>
+      </c>
+      <c r="F707" t="n">
+        <v>71.3</v>
+      </c>
+    </row>
+    <row r="708">
+      <c r="A708" s="2" t="n">
+        <v>46087</v>
+      </c>
+      <c r="B708" t="inlineStr">
+        <is>
+          <t>牛前八件套</t>
+        </is>
+      </c>
+      <c r="C708" t="n">
+        <v>57.04</v>
+      </c>
+      <c r="D708" t="n">
+        <v>57.25</v>
+      </c>
+      <c r="E708" t="n">
+        <v>56.79</v>
+      </c>
+      <c r="F708" t="n">
+        <v>57.2</v>
+      </c>
+    </row>
+    <row r="709">
+      <c r="A709" s="2" t="n">
+        <v>46087</v>
+      </c>
+      <c r="B709" t="inlineStr">
+        <is>
+          <t>龟排腱</t>
+        </is>
+      </c>
+      <c r="C709" t="n">
+        <v>71.37</v>
+      </c>
+      <c r="D709" t="n">
+        <v>71.62</v>
+      </c>
+      <c r="E709" t="n">
+        <v>70.95</v>
+      </c>
+      <c r="F709" t="n">
+        <v>71.3</v>
+      </c>
+    </row>
+    <row r="710">
+      <c r="A710" s="2" t="n">
+        <v>46090</v>
+      </c>
+      <c r="B710" t="inlineStr">
+        <is>
+          <t>牛前八件套</t>
+        </is>
+      </c>
+      <c r="C710" t="n">
+        <v>58.17</v>
+      </c>
+      <c r="D710" t="n">
+        <v>58.65</v>
+      </c>
+      <c r="E710" t="n">
+        <v>58.15</v>
+      </c>
+      <c r="F710" t="n">
+        <v>58.5</v>
+      </c>
+    </row>
+    <row r="711">
+      <c r="A711" s="2" t="n">
+        <v>46090</v>
+      </c>
+      <c r="B711" t="inlineStr">
+        <is>
+          <t>龟排腱</t>
+        </is>
+      </c>
+      <c r="C711" t="n">
+        <v>70.91</v>
+      </c>
+      <c r="D711" t="n">
+        <v>71.68000000000001</v>
+      </c>
+      <c r="E711" t="n">
+        <v>70.81999999999999</v>
+      </c>
+      <c r="F711" t="n">
+        <v>71.3</v>
+      </c>
+    </row>
+    <row r="712">
+      <c r="A712" s="2" t="n">
+        <v>46091</v>
+      </c>
+      <c r="B712" t="inlineStr">
+        <is>
+          <t>牛前八件套</t>
+        </is>
+      </c>
+      <c r="C712" t="n">
+        <v>58.28</v>
+      </c>
+      <c r="D712" t="n">
+        <v>58.64</v>
+      </c>
+      <c r="E712" t="n">
+        <v>58.07</v>
+      </c>
+      <c r="F712" t="n">
+        <v>58.5</v>
+      </c>
+    </row>
+    <row r="713">
+      <c r="A713" s="2" t="n">
+        <v>46091</v>
+      </c>
+      <c r="B713" t="inlineStr">
+        <is>
+          <t>龟排腱</t>
+        </is>
+      </c>
+      <c r="C713" t="n">
+        <v>71.05</v>
+      </c>
+      <c r="D713" t="n">
+        <v>71.7</v>
+      </c>
+      <c r="E713" t="n">
+        <v>70.81999999999999</v>
+      </c>
+      <c r="F713" t="n">
+        <v>71.3</v>
+      </c>
+    </row>
+    <row r="714">
+      <c r="A714" s="2" t="n">
+        <v>46092</v>
+      </c>
+      <c r="B714" t="inlineStr">
+        <is>
+          <t>牛前八件套</t>
+        </is>
+      </c>
+      <c r="C714" t="n">
+        <v>58.28</v>
+      </c>
+      <c r="D714" t="n">
+        <v>58.53</v>
+      </c>
+      <c r="E714" t="n">
+        <v>57.99</v>
+      </c>
+      <c r="F714" t="n">
+        <v>58.2</v>
+      </c>
+    </row>
+    <row r="715">
+      <c r="A715" s="2" t="n">
+        <v>46092</v>
+      </c>
+      <c r="B715" t="inlineStr">
+        <is>
+          <t>龟排腱</t>
+        </is>
+      </c>
+      <c r="C715" t="n">
+        <v>71.8</v>
+      </c>
+      <c r="D715" t="n">
+        <v>72.03</v>
+      </c>
+      <c r="E715" t="n">
+        <v>71</v>
+      </c>
+      <c r="F715" t="n">
+        <v>71.3</v>
+      </c>
+    </row>
+    <row r="716">
+      <c r="A716" s="2" t="n">
+        <v>46093</v>
+      </c>
+      <c r="B716" t="inlineStr">
+        <is>
+          <t>牛前八件套</t>
+        </is>
+      </c>
+      <c r="C716" t="n">
+        <v>58.1</v>
+      </c>
+      <c r="D716" t="n">
+        <v>58.31</v>
+      </c>
+      <c r="E716" t="n">
+        <v>57.77</v>
+      </c>
+      <c r="F716" t="n">
+        <v>58.1</v>
+      </c>
+    </row>
+    <row r="717">
+      <c r="A717" s="2" t="n">
+        <v>46093</v>
+      </c>
+      <c r="B717" t="inlineStr">
+        <is>
+          <t>龟排腱</t>
+        </is>
+      </c>
+      <c r="C717" t="n">
+        <v>71.78</v>
+      </c>
+      <c r="D717" t="n">
+        <v>72</v>
+      </c>
+      <c r="E717" t="n">
+        <v>71.69</v>
+      </c>
+      <c r="F717" t="n">
+        <v>71.8</v>
+      </c>
+    </row>
+    <row r="718">
+      <c r="A718" s="2" t="n">
+        <v>46094</v>
+      </c>
+      <c r="B718" t="inlineStr">
+        <is>
+          <t>牛前八件套</t>
+        </is>
+      </c>
+      <c r="C718" t="n">
+        <v>57.79</v>
+      </c>
+      <c r="D718" t="n">
+        <v>58.01</v>
+      </c>
+      <c r="E718" t="n">
+        <v>57.49</v>
+      </c>
+      <c r="F718" t="n">
+        <v>57.7</v>
+      </c>
+    </row>
+    <row r="719">
+      <c r="A719" s="2" t="n">
+        <v>46094</v>
+      </c>
+      <c r="B719" t="inlineStr">
+        <is>
+          <t>龟排腱</t>
+        </is>
+      </c>
+      <c r="C719" t="n">
+        <v>71.43000000000001</v>
+      </c>
+      <c r="D719" t="n">
+        <v>72.31999999999999</v>
+      </c>
+      <c r="E719" t="n">
+        <v>71.29000000000001</v>
+      </c>
+      <c r="F719" t="n">
+        <v>71.8</v>
+      </c>
+    </row>
+    <row r="720">
+      <c r="A720" s="2" t="n">
+        <v>46095</v>
+      </c>
+      <c r="B720" t="inlineStr">
+        <is>
+          <t>牛前八件套</t>
+        </is>
+      </c>
+      <c r="C720" t="n">
+        <v>57.73</v>
+      </c>
+      <c r="D720" t="n">
+        <v>57.85</v>
+      </c>
+      <c r="E720" t="n">
+        <v>57.69</v>
+      </c>
+      <c r="F720" t="n">
+        <v>57.7</v>
+      </c>
+    </row>
+    <row r="721">
+      <c r="A721" s="2" t="n">
+        <v>46095</v>
+      </c>
+      <c r="B721" t="inlineStr">
+        <is>
+          <t>龟排腱</t>
+        </is>
+      </c>
+      <c r="C721" t="n">
+        <v>72.36</v>
+      </c>
+      <c r="D721" t="n">
+        <v>72.59</v>
+      </c>
+      <c r="E721" t="n">
+        <v>71.37</v>
+      </c>
+      <c r="F721" t="n">
+        <v>71.8</v>
+      </c>
+    </row>
+    <row r="722">
+      <c r="A722" s="2" t="n">
+        <v>46097</v>
+      </c>
+      <c r="B722" t="inlineStr">
+        <is>
+          <t>牛前八件套</t>
+        </is>
+      </c>
+      <c r="C722" t="n">
+        <v>57.5</v>
+      </c>
+      <c r="D722" t="n">
+        <v>57.73</v>
+      </c>
+      <c r="E722" t="n">
+        <v>57.2</v>
+      </c>
+      <c r="F722" t="n">
+        <v>57.5</v>
+      </c>
+    </row>
+    <row r="723">
+      <c r="A723" s="2" t="n">
+        <v>46097</v>
+      </c>
+      <c r="B723" t="inlineStr">
+        <is>
+          <t>龟排腱</t>
+        </is>
+      </c>
+      <c r="C723" t="n">
+        <v>71.55</v>
+      </c>
+      <c r="D723" t="n">
+        <v>72.2</v>
+      </c>
+      <c r="E723" t="n">
+        <v>71.31999999999999</v>
+      </c>
+      <c r="F723" t="n">
+        <v>71.8</v>
+      </c>
+    </row>
+    <row r="724">
+      <c r="A724" s="2" t="n">
+        <v>46098</v>
+      </c>
+      <c r="B724" t="inlineStr">
+        <is>
+          <t>牛前八件套</t>
+        </is>
+      </c>
+      <c r="C724" t="n">
+        <v>57.57</v>
+      </c>
+      <c r="D724" t="n">
+        <v>57.93</v>
+      </c>
+      <c r="E724" t="n">
+        <v>57.55</v>
+      </c>
+      <c r="F724" t="n">
+        <v>57.6</v>
+      </c>
+    </row>
+    <row r="725">
+      <c r="A725" s="2" t="n">
+        <v>46098</v>
+      </c>
+      <c r="B725" t="inlineStr">
+        <is>
+          <t>龟排腱</t>
+        </is>
+      </c>
+      <c r="C725" t="n">
+        <v>72.3</v>
+      </c>
+      <c r="D725" t="n">
+        <v>72.54000000000001</v>
+      </c>
+      <c r="E725" t="n">
+        <v>71.48999999999999</v>
+      </c>
+      <c r="F725" t="n">
+        <v>71.8</v>
+      </c>
+    </row>
+    <row r="726">
+      <c r="A726" s="2" t="n">
+        <v>46099</v>
+      </c>
+      <c r="B726" t="inlineStr">
+        <is>
+          <t>牛前八件套</t>
+        </is>
+      </c>
+      <c r="C726" t="n">
+        <v>57.77</v>
+      </c>
+      <c r="D726" t="n">
+        <v>57.85</v>
+      </c>
+      <c r="E726" t="n">
+        <v>57.52</v>
+      </c>
+      <c r="F726" t="n">
+        <v>57.8</v>
+      </c>
+    </row>
+    <row r="727">
+      <c r="A727" s="2" t="n">
+        <v>46099</v>
+      </c>
+      <c r="B727" t="inlineStr">
+        <is>
+          <t>龟排腱</t>
+        </is>
+      </c>
+      <c r="C727" t="n">
+        <v>71.22</v>
+      </c>
+      <c r="D727" t="n">
+        <v>72</v>
+      </c>
+      <c r="E727" t="n">
+        <v>71.12</v>
+      </c>
+      <c r="F727" t="n">
+        <v>71.8</v>
+      </c>
+    </row>
+    <row r="728">
+      <c r="A728" s="2" t="n">
+        <v>46100</v>
+      </c>
+      <c r="B728" t="inlineStr">
+        <is>
+          <t>牛前八件套</t>
+        </is>
+      </c>
+      <c r="C728" t="n">
+        <v>57.94</v>
+      </c>
+      <c r="D728" t="n">
+        <v>58.04</v>
+      </c>
+      <c r="E728" t="n">
+        <v>57.77</v>
+      </c>
+      <c r="F728" t="n">
+        <v>57.8</v>
+      </c>
+    </row>
+    <row r="729">
+      <c r="A729" s="2" t="n">
+        <v>46100</v>
+      </c>
+      <c r="B729" t="inlineStr">
+        <is>
+          <t>龟排腱</t>
+        </is>
+      </c>
+      <c r="C729" t="n">
+        <v>71.43000000000001</v>
+      </c>
+      <c r="D729" t="n">
+        <v>72.31999999999999</v>
+      </c>
+      <c r="E729" t="n">
+        <v>71.29000000000001</v>
+      </c>
+      <c r="F729" t="n">
+        <v>71.8</v>
+      </c>
+    </row>
+    <row r="730">
+      <c r="A730" s="2" t="n">
+        <v>46101</v>
+      </c>
+      <c r="B730" t="inlineStr">
+        <is>
+          <t>牛前八件套</t>
+        </is>
+      </c>
+      <c r="C730" t="n">
+        <v>57.58</v>
+      </c>
+      <c r="D730" t="n">
+        <v>57.94</v>
+      </c>
+      <c r="E730" t="n">
+        <v>57.37</v>
+      </c>
+      <c r="F730" t="n">
+        <v>57.8</v>
+      </c>
+    </row>
+    <row r="731">
+      <c r="A731" s="2" t="n">
+        <v>46101</v>
+      </c>
+      <c r="B731" t="inlineStr">
+        <is>
+          <t>龟排腱</t>
+        </is>
+      </c>
+      <c r="C731" t="n">
+        <v>72.36</v>
+      </c>
+      <c r="D731" t="n">
+        <v>72.59</v>
+      </c>
+      <c r="E731" t="n">
+        <v>71.37</v>
+      </c>
+      <c r="F731" t="n">
+        <v>71.8</v>
+      </c>
+    </row>
+    <row r="732">
+      <c r="A732" s="2" t="n">
+        <v>46104</v>
+      </c>
+      <c r="B732" t="inlineStr">
+        <is>
+          <t>牛前八件套</t>
+        </is>
+      </c>
+      <c r="C732" t="n">
+        <v>57.58</v>
+      </c>
+      <c r="D732" t="n">
+        <v>57.83</v>
+      </c>
+      <c r="E732" t="n">
+        <v>57.3</v>
+      </c>
+      <c r="F732" t="n">
+        <v>57.5</v>
+      </c>
+    </row>
+    <row r="733">
+      <c r="A733" s="2" t="n">
+        <v>46104</v>
+      </c>
+      <c r="B733" t="inlineStr">
+        <is>
+          <t>龟排腱</t>
+        </is>
+      </c>
+      <c r="C733" t="n">
+        <v>71.8</v>
+      </c>
+      <c r="D733" t="n">
+        <v>72.01000000000001</v>
+      </c>
+      <c r="E733" t="n">
+        <v>71.53</v>
+      </c>
+      <c r="F733" t="n">
+        <v>71.8</v>
+      </c>
+    </row>
+    <row r="734">
+      <c r="A734" s="2" t="n">
+        <v>46105</v>
+      </c>
+      <c r="B734" t="inlineStr">
+        <is>
+          <t>牛前八件套</t>
+        </is>
+      </c>
+      <c r="C734" t="n">
+        <v>57.31</v>
+      </c>
+      <c r="D734" t="n">
+        <v>57.51</v>
+      </c>
+      <c r="E734" t="n">
+        <v>56.97</v>
+      </c>
+      <c r="F734" t="n">
+        <v>57.3</v>
+      </c>
+    </row>
+    <row r="735">
+      <c r="A735" s="2" t="n">
+        <v>46105</v>
+      </c>
+      <c r="B735" t="inlineStr">
+        <is>
+          <t>龟排腱</t>
+        </is>
+      </c>
+      <c r="C735" t="n">
+        <v>71.34</v>
+      </c>
+      <c r="D735" t="n">
+        <v>71.59999999999999</v>
+      </c>
+      <c r="E735" t="n">
+        <v>71.15000000000001</v>
+      </c>
+      <c r="F735" t="n">
+        <v>71.3</v>
+      </c>
+    </row>
+    <row r="736">
+      <c r="A736" s="2" t="n">
+        <v>46106</v>
+      </c>
+      <c r="B736" t="inlineStr">
+        <is>
+          <t>牛前八件套</t>
+        </is>
+      </c>
+      <c r="C736" t="n">
+        <v>57.14</v>
+      </c>
+      <c r="D736" t="n">
+        <v>57.37</v>
+      </c>
+      <c r="E736" t="n">
+        <v>56.89</v>
+      </c>
+      <c r="F736" t="n">
+        <v>57.1</v>
+      </c>
+    </row>
+    <row r="737">
+      <c r="A737" s="2" t="n">
+        <v>46106</v>
+      </c>
+      <c r="B737" t="inlineStr">
+        <is>
+          <t>龟排腱</t>
+        </is>
+      </c>
+      <c r="C737" t="n">
+        <v>70.62</v>
+      </c>
+      <c r="D737" t="n">
+        <v>71.65000000000001</v>
+      </c>
+      <c r="E737" t="n">
+        <v>70.56</v>
+      </c>
+      <c r="F737" t="n">
+        <v>71.3</v>
+      </c>
+    </row>
+    <row r="738">
+      <c r="A738" s="2" t="n">
+        <v>46107</v>
+      </c>
+      <c r="B738" t="inlineStr">
+        <is>
+          <t>牛前八件套</t>
+        </is>
+      </c>
+      <c r="C738" t="n">
+        <v>57.13</v>
+      </c>
+      <c r="D738" t="n">
+        <v>57.25</v>
+      </c>
+      <c r="E738" t="n">
+        <v>57.09</v>
+      </c>
+      <c r="F738" t="n">
+        <v>57.1</v>
+      </c>
+    </row>
+    <row r="739">
+      <c r="A739" s="2" t="n">
+        <v>46107</v>
+      </c>
+      <c r="B739" t="inlineStr">
+        <is>
+          <t>龟排腱</t>
+        </is>
+      </c>
+      <c r="C739" t="n">
+        <v>71.93000000000001</v>
+      </c>
+      <c r="D739" t="n">
+        <v>72.27</v>
+      </c>
+      <c r="E739" t="n">
+        <v>70.81</v>
+      </c>
+      <c r="F739" t="n">
+        <v>71.3</v>
+      </c>
+    </row>
+    <row r="740">
+      <c r="A740" s="2" t="n">
+        <v>46108</v>
+      </c>
+      <c r="B740" t="inlineStr">
+        <is>
+          <t>牛前八件套</t>
+        </is>
+      </c>
+      <c r="C740" t="n">
+        <v>57.29</v>
+      </c>
+      <c r="D740" t="n">
+        <v>57.31</v>
+      </c>
+      <c r="E740" t="n">
+        <v>57.11</v>
+      </c>
+      <c r="F740" t="n">
+        <v>57.3</v>
+      </c>
+    </row>
+    <row r="741">
+      <c r="A741" s="2" t="n">
+        <v>46108</v>
+      </c>
+      <c r="B741" t="inlineStr">
+        <is>
+          <t>龟排腱</t>
+        </is>
+      </c>
+      <c r="C741" t="n">
+        <v>71.11</v>
+      </c>
+      <c r="D741" t="n">
+        <v>71.31</v>
+      </c>
+      <c r="E741" t="n">
+        <v>70.78</v>
+      </c>
+      <c r="F741" t="n">
+        <v>71.3</v>
+      </c>
+    </row>
+    <row r="742">
+      <c r="A742" s="2" t="n">
+        <v>46111</v>
+      </c>
+      <c r="B742" t="inlineStr">
+        <is>
+          <t>牛前八件套</t>
+        </is>
+      </c>
+      <c r="C742" t="n">
+        <v>57.09</v>
+      </c>
+      <c r="D742" t="n">
+        <v>57.52</v>
+      </c>
+      <c r="E742" t="n">
+        <v>56.83</v>
+      </c>
+      <c r="F742" t="n">
+        <v>57.3</v>
+      </c>
+    </row>
+    <row r="743">
+      <c r="A743" s="2" t="n">
+        <v>46111</v>
+      </c>
+      <c r="B743" t="inlineStr">
+        <is>
+          <t>龟排腱</t>
+        </is>
+      </c>
+      <c r="C743" t="n">
+        <v>71.2</v>
+      </c>
+      <c r="D743" t="n">
+        <v>71.81999999999999</v>
+      </c>
+      <c r="E743" t="n">
+        <v>70.84999999999999</v>
+      </c>
+      <c r="F743" t="n">
+        <v>71.3</v>
+      </c>
+    </row>
+    <row r="744">
+      <c r="A744" s="2" t="n">
+        <v>46112</v>
+      </c>
+      <c r="B744" t="inlineStr">
+        <is>
+          <t>牛前八件套</t>
+        </is>
+      </c>
+      <c r="C744" t="n">
+        <v>57.12</v>
+      </c>
+      <c r="D744" t="n">
+        <v>57.24</v>
+      </c>
+      <c r="E744" t="n">
+        <v>56.78</v>
+      </c>
+      <c r="F744" t="n">
+        <v>57.1</v>
+      </c>
+    </row>
+    <row r="745">
+      <c r="A745" s="2" t="n">
+        <v>46112</v>
+      </c>
+      <c r="B745" t="inlineStr">
+        <is>
+          <t>龟排腱</t>
+        </is>
+      </c>
+      <c r="C745" t="n">
+        <v>71.8</v>
+      </c>
+      <c r="D745" t="n">
+        <v>71.91</v>
+      </c>
+      <c r="E745" t="n">
+        <v>71.09</v>
+      </c>
+      <c r="F745" t="n">
+        <v>71.3</v>
+      </c>
+    </row>
+    <row r="746">
+      <c r="A746" s="2" t="n">
+        <v>46113</v>
+      </c>
+      <c r="B746" t="inlineStr">
+        <is>
+          <t>牛前八件套</t>
+        </is>
+      </c>
+      <c r="C746" t="n">
+        <v>56.69</v>
+      </c>
+      <c r="D746" t="n">
+        <v>57.44</v>
+      </c>
+      <c r="E746" t="n">
+        <v>56.67</v>
+      </c>
+      <c r="F746" t="n">
+        <v>57.1</v>
+      </c>
+    </row>
+    <row r="747">
+      <c r="A747" s="2" t="n">
+        <v>46113</v>
+      </c>
+      <c r="B747" t="inlineStr">
+        <is>
+          <t>龟排腱</t>
+        </is>
+      </c>
+      <c r="C747" t="n">
+        <v>71.84999999999999</v>
+      </c>
+      <c r="D747" t="n">
+        <v>72.13</v>
+      </c>
+      <c r="E747" t="n">
+        <v>70.95999999999999</v>
+      </c>
+      <c r="F747" t="n">
+        <v>71.3</v>
+      </c>
+    </row>
+    <row r="748">
+      <c r="A748" s="2" t="n">
+        <v>46114</v>
+      </c>
+      <c r="B748" t="inlineStr">
+        <is>
+          <t>牛前八件套</t>
+        </is>
+      </c>
+      <c r="C748" t="n">
+        <v>57.66</v>
+      </c>
+      <c r="D748" t="n">
+        <v>57.88</v>
+      </c>
+      <c r="E748" t="n">
+        <v>57.01</v>
+      </c>
+      <c r="F748" t="n">
+        <v>57.1</v>
+      </c>
+    </row>
+    <row r="749">
+      <c r="A749" s="2" t="n">
+        <v>46114</v>
+      </c>
+      <c r="B749" t="inlineStr">
+        <is>
+          <t>龟排腱</t>
+        </is>
+      </c>
+      <c r="C749" t="n">
+        <v>70.70999999999999</v>
+      </c>
+      <c r="D749" t="n">
+        <v>71.39</v>
+      </c>
+      <c r="E749" t="n">
+        <v>70.39</v>
+      </c>
+      <c r="F749" t="n">
+        <v>71.3</v>
+      </c>
+    </row>
+    <row r="750">
+      <c r="A750" s="2" t="n">
+        <v>46115</v>
+      </c>
+      <c r="B750" t="inlineStr">
+        <is>
+          <t>牛前八件套</t>
+        </is>
+      </c>
+      <c r="C750" t="n">
+        <v>56.54</v>
+      </c>
+      <c r="D750" t="n">
+        <v>57.45</v>
+      </c>
+      <c r="E750" t="n">
+        <v>56.34</v>
+      </c>
+      <c r="F750" t="n">
+        <v>57.1</v>
+      </c>
+    </row>
+    <row r="751">
+      <c r="A751" s="2" t="n">
+        <v>46115</v>
+      </c>
+      <c r="B751" t="inlineStr">
+        <is>
+          <t>龟排腱</t>
+        </is>
+      </c>
+      <c r="C751" t="n">
+        <v>71.45</v>
+      </c>
+      <c r="D751" t="n">
+        <v>71.45999999999999</v>
+      </c>
+      <c r="E751" t="n">
+        <v>71.25</v>
+      </c>
+      <c r="F751" t="n">
+        <v>71.3</v>
+      </c>
+    </row>
+    <row r="752">
+      <c r="A752" s="2" t="n">
+        <v>46118</v>
+      </c>
+      <c r="B752" t="inlineStr">
+        <is>
+          <t>牛前八件套</t>
+        </is>
+      </c>
+      <c r="C752" t="n">
+        <v>57.24</v>
+      </c>
+      <c r="D752" t="n">
+        <v>57.63</v>
+      </c>
+      <c r="E752" t="n">
+        <v>57.22</v>
+      </c>
+      <c r="F752" t="n">
+        <v>57.3</v>
+      </c>
+    </row>
+    <row r="753">
+      <c r="A753" s="2" t="n">
+        <v>46118</v>
+      </c>
+      <c r="B753" t="inlineStr">
+        <is>
+          <t>龟排腱</t>
+        </is>
+      </c>
+      <c r="C753" t="n">
+        <v>71.53</v>
+      </c>
+      <c r="D753" t="n">
+        <v>71.53</v>
+      </c>
+      <c r="E753" t="n">
+        <v>71.20999999999999</v>
+      </c>
+      <c r="F753" t="n">
+        <v>71.3</v>
+      </c>
+    </row>
+    <row r="754">
+      <c r="A754" s="2" t="n">
+        <v>46119</v>
+      </c>
+      <c r="B754" t="inlineStr">
+        <is>
+          <t>牛前八件套</t>
+        </is>
+      </c>
+      <c r="C754" t="n">
+        <v>57.39</v>
+      </c>
+      <c r="D754" t="n">
+        <v>57.45</v>
+      </c>
+      <c r="E754" t="n">
+        <v>57.14</v>
+      </c>
+      <c r="F754" t="n">
+        <v>57.4</v>
+      </c>
+    </row>
+    <row r="755">
+      <c r="A755" s="2" t="n">
+        <v>46119</v>
+      </c>
+      <c r="B755" t="inlineStr">
+        <is>
+          <t>龟排腱</t>
+        </is>
+      </c>
+      <c r="C755" t="n">
+        <v>71.37</v>
+      </c>
+      <c r="D755" t="n">
+        <v>71.62</v>
+      </c>
+      <c r="E755" t="n">
+        <v>70.95</v>
+      </c>
+      <c r="F755" t="n">
+        <v>71.3</v>
+      </c>
+    </row>
+    <row r="756">
+      <c r="A756" s="2" t="n">
+        <v>46120</v>
+      </c>
+      <c r="B756" t="inlineStr">
+        <is>
+          <t>牛前八件套</t>
+        </is>
+      </c>
+      <c r="C756" t="n">
+        <v>57.54</v>
+      </c>
+      <c r="D756" t="n">
+        <v>57.64</v>
+      </c>
+      <c r="E756" t="n">
+        <v>57.37</v>
+      </c>
+      <c r="F756" t="n">
+        <v>57.4</v>
+      </c>
+    </row>
+    <row r="757">
+      <c r="A757" s="2" t="n">
+        <v>46120</v>
+      </c>
+      <c r="B757" t="inlineStr">
+        <is>
+          <t>龟排腱</t>
+        </is>
+      </c>
+      <c r="C757" t="n">
+        <v>70.91</v>
+      </c>
+      <c r="D757" t="n">
+        <v>71.68000000000001</v>
+      </c>
+      <c r="E757" t="n">
+        <v>70.81999999999999</v>
+      </c>
+      <c r="F757" t="n">
+        <v>71.3</v>
+      </c>
+    </row>
+    <row r="758">
+      <c r="A758" s="2" t="n">
+        <v>46121</v>
+      </c>
+      <c r="B758" t="inlineStr">
+        <is>
+          <t>牛前八件套</t>
+        </is>
+      </c>
+      <c r="C758" t="n">
+        <v>57.49</v>
+      </c>
+      <c r="D758" t="n">
+        <v>57.64</v>
+      </c>
+      <c r="E758" t="n">
+        <v>57.28</v>
+      </c>
+      <c r="F758" t="n">
+        <v>57.5</v>
+      </c>
+    </row>
+    <row r="759">
+      <c r="A759" s="2" t="n">
+        <v>46121</v>
+      </c>
+      <c r="B759" t="inlineStr">
+        <is>
+          <t>龟排腱</t>
+        </is>
+      </c>
+      <c r="C759" t="n">
+        <v>71.05</v>
+      </c>
+      <c r="D759" t="n">
+        <v>71.7</v>
+      </c>
+      <c r="E759" t="n">
+        <v>70.81999999999999</v>
+      </c>
+      <c r="F759" t="n">
+        <v>71.3</v>
+      </c>
+    </row>
+    <row r="760">
+      <c r="A760" s="2" t="n">
+        <v>46122</v>
+      </c>
+      <c r="B760" t="inlineStr">
+        <is>
+          <t>牛前八件套</t>
+        </is>
+      </c>
+      <c r="C760" t="n">
+        <v>57.57</v>
+      </c>
+      <c r="D760" t="n">
+        <v>57.98</v>
+      </c>
+      <c r="E760" t="n">
+        <v>57.44</v>
+      </c>
+      <c r="F760" t="n">
+        <v>57.6</v>
+      </c>
+    </row>
+    <row r="761">
+      <c r="A761" s="2" t="n">
+        <v>46122</v>
+      </c>
+      <c r="B761" t="inlineStr">
+        <is>
+          <t>龟排腱</t>
+        </is>
+      </c>
+      <c r="C761" t="n">
+        <v>71.8</v>
+      </c>
+      <c r="D761" t="n">
+        <v>72.03</v>
+      </c>
+      <c r="E761" t="n">
+        <v>71</v>
+      </c>
+      <c r="F761" t="n">
+        <v>71.3</v>
+      </c>
+    </row>
+    <row r="762">
+      <c r="A762" s="2" t="n">
+        <v>46125</v>
+      </c>
+      <c r="B762" t="inlineStr">
+        <is>
+          <t>牛前八件套</t>
+        </is>
+      </c>
+      <c r="C762" t="n">
+        <v>57.79</v>
+      </c>
+      <c r="D762" t="n">
+        <v>58.11</v>
+      </c>
+      <c r="E762" t="n">
+        <v>57.57</v>
+      </c>
+      <c r="F762" t="n">
+        <v>57.8</v>
+      </c>
+    </row>
+    <row r="763">
+      <c r="A763" s="2" t="n">
+        <v>46125</v>
+      </c>
+      <c r="B763" t="inlineStr">
+        <is>
+          <t>龟排腱</t>
+        </is>
+      </c>
+      <c r="C763" t="n">
+        <v>70.72</v>
+      </c>
+      <c r="D763" t="n">
+        <v>71.5</v>
+      </c>
+      <c r="E763" t="n">
+        <v>70.63</v>
+      </c>
+      <c r="F763" t="n">
+        <v>71.3</v>
+      </c>
+    </row>
+    <row r="764">
+      <c r="A764" s="2" t="n">
+        <v>46126</v>
+      </c>
+      <c r="B764" t="inlineStr">
+        <is>
+          <t>牛前八件套</t>
+        </is>
+      </c>
+      <c r="C764" t="n">
+        <v>57.87</v>
+      </c>
+      <c r="D764" t="n">
+        <v>58.09</v>
+      </c>
+      <c r="E764" t="n">
+        <v>57.59</v>
+      </c>
+      <c r="F764" t="n">
+        <v>57.8</v>
+      </c>
+    </row>
+    <row r="765">
+      <c r="A765" s="2" t="n">
+        <v>46126</v>
+      </c>
+      <c r="B765" t="inlineStr">
+        <is>
+          <t>龟排腱</t>
+        </is>
+      </c>
+      <c r="C765" t="n">
+        <v>70.93000000000001</v>
+      </c>
+      <c r="D765" t="n">
+        <v>71.81999999999999</v>
+      </c>
+      <c r="E765" t="n">
+        <v>70.8</v>
+      </c>
+      <c r="F765" t="n">
+        <v>71.3</v>
+      </c>
+    </row>
+    <row r="766">
+      <c r="A766" s="2" t="n">
+        <v>46127</v>
+      </c>
+      <c r="B766" t="inlineStr">
+        <is>
+          <t>牛前八件套</t>
+        </is>
+      </c>
+      <c r="C766" t="n">
+        <v>57.96</v>
+      </c>
+      <c r="D766" t="n">
+        <v>58.19</v>
+      </c>
+      <c r="E766" t="n">
+        <v>57.95</v>
+      </c>
+      <c r="F766" t="n">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="767">
+      <c r="A767" s="2" t="n">
+        <v>46127</v>
+      </c>
+      <c r="B767" t="inlineStr">
+        <is>
+          <t>龟排腱</t>
+        </is>
+      </c>
+      <c r="C767" t="n">
+        <v>71.86</v>
+      </c>
+      <c r="D767" t="n">
+        <v>72.09</v>
+      </c>
+      <c r="E767" t="n">
+        <v>70.87</v>
+      </c>
+      <c r="F767" t="n">
+        <v>71.3</v>
+      </c>
+    </row>
+    <row r="768">
+      <c r="A768" s="2" t="n">
+        <v>46128</v>
+      </c>
+      <c r="B768" t="inlineStr">
+        <is>
+          <t>牛前八件套</t>
+        </is>
+      </c>
+      <c r="C768" t="n">
+        <v>58.09</v>
+      </c>
+      <c r="D768" t="n">
+        <v>58.45</v>
+      </c>
+      <c r="E768" t="n">
+        <v>58.07</v>
+      </c>
+      <c r="F768" t="n">
+        <v>58.1</v>
+      </c>
+    </row>
+    <row r="769">
+      <c r="A769" s="2" t="n">
+        <v>46128</v>
+      </c>
+      <c r="B769" t="inlineStr">
+        <is>
+          <t>龟排腱</t>
+        </is>
+      </c>
+      <c r="C769" t="n">
+        <v>71.84999999999999</v>
+      </c>
+      <c r="D769" t="n">
+        <v>72.13</v>
+      </c>
+      <c r="E769" t="n">
+        <v>70.95999999999999</v>
+      </c>
+      <c r="F769" t="n">
+        <v>71.3</v>
+      </c>
+    </row>
+    <row r="770">
+      <c r="A770" s="2" t="n">
+        <v>46129</v>
+      </c>
+      <c r="B770" t="inlineStr">
+        <is>
+          <t>牛前八件套</t>
+        </is>
+      </c>
+      <c r="C770" t="n">
+        <v>58.67</v>
+      </c>
+      <c r="D770" t="n">
+        <v>58.89</v>
+      </c>
+      <c r="E770" t="n">
+        <v>58.01</v>
+      </c>
+      <c r="F770" t="n">
+        <v>58.1</v>
+      </c>
+    </row>
+    <row r="771">
+      <c r="A771" s="2" t="n">
+        <v>46129</v>
+      </c>
+      <c r="B771" t="inlineStr">
+        <is>
+          <t>龟排腱</t>
+        </is>
+      </c>
+      <c r="C771" t="n">
+        <v>71.40000000000001</v>
+      </c>
+      <c r="D771" t="n">
+        <v>71.48999999999999</v>
+      </c>
+      <c r="E771" t="n">
+        <v>71.08</v>
+      </c>
+      <c r="F771" t="n">
+        <v>71.40000000000001</v>
+      </c>
+    </row>
+    <row r="772">
+      <c r="A772" s="2" t="n">
+        <v>46132</v>
+      </c>
+      <c r="B772" t="inlineStr">
+        <is>
+          <t>牛前八件套</t>
+        </is>
+      </c>
+      <c r="C772" t="n">
+        <v>57.53</v>
+      </c>
+      <c r="D772" t="n">
+        <v>58.46</v>
+      </c>
+      <c r="E772" t="n">
+        <v>57.32</v>
+      </c>
+      <c r="F772" t="n">
+        <v>58.1</v>
+      </c>
+    </row>
+    <row r="773">
+      <c r="A773" s="2" t="n">
+        <v>46132</v>
+      </c>
+      <c r="B773" t="inlineStr">
+        <is>
+          <t>龟排腱</t>
+        </is>
+      </c>
+      <c r="C773" t="n">
+        <v>71.55</v>
+      </c>
+      <c r="D773" t="n">
+        <v>71.56</v>
+      </c>
+      <c r="E773" t="n">
+        <v>71.34999999999999</v>
+      </c>
+      <c r="F773" t="n">
+        <v>71.40000000000001</v>
+      </c>
+    </row>
+    <row r="774">
+      <c r="A774" s="2" t="n">
+        <v>46133</v>
+      </c>
+      <c r="B774" t="inlineStr">
+        <is>
+          <t>牛前八件套</t>
+        </is>
+      </c>
+      <c r="C774" t="n">
+        <v>58.37</v>
+      </c>
+      <c r="D774" t="n">
+        <v>58.59</v>
+      </c>
+      <c r="E774" t="n">
+        <v>58.07</v>
+      </c>
+      <c r="F774" t="n">
+        <v>58.1</v>
+      </c>
+    </row>
+    <row r="775">
+      <c r="A775" s="2" t="n">
+        <v>46133</v>
+      </c>
+      <c r="B775" t="inlineStr">
+        <is>
+          <t>龟排腱</t>
+        </is>
+      </c>
+      <c r="C775" t="n">
+        <v>71.47</v>
+      </c>
+      <c r="D775" t="n">
+        <v>71.5</v>
+      </c>
+      <c r="E775" t="n">
+        <v>71.42</v>
+      </c>
+      <c r="F775" t="n">
+        <v>71.5</v>
+      </c>
+    </row>
+    <row r="776">
+      <c r="A776" s="2" t="n">
+        <v>46134</v>
+      </c>
+      <c r="B776" t="inlineStr">
+        <is>
+          <t>牛前八件套</t>
+        </is>
+      </c>
+      <c r="C776" t="n">
+        <v>58.36</v>
+      </c>
+      <c r="D776" t="n">
+        <v>58.45</v>
+      </c>
+      <c r="E776" t="n">
+        <v>58.1</v>
+      </c>
+      <c r="F776" t="n">
+        <v>58.4</v>
+      </c>
+    </row>
+    <row r="777">
+      <c r="A777" s="2" t="n">
+        <v>46134</v>
+      </c>
+      <c r="B777" t="inlineStr">
+        <is>
+          <t>龟排腱</t>
+        </is>
+      </c>
+      <c r="C777" t="n">
+        <v>71.56999999999999</v>
+      </c>
+      <c r="D777" t="n">
+        <v>71.81999999999999</v>
+      </c>
+      <c r="E777" t="n">
+        <v>71.15000000000001</v>
+      </c>
+      <c r="F777" t="n">
+        <v>71.5</v>
+      </c>
+    </row>
+    <row r="778">
+      <c r="A778" s="2" t="n">
+        <v>46135</v>
+      </c>
+      <c r="B778" t="inlineStr">
+        <is>
+          <t>牛前八件套</t>
+        </is>
+      </c>
+      <c r="C778" t="n">
+        <v>58.54</v>
+      </c>
+      <c r="D778" t="n">
+        <v>58.64</v>
+      </c>
+      <c r="E778" t="n">
+        <v>58.37</v>
+      </c>
+      <c r="F778" t="n">
+        <v>58.4</v>
+      </c>
+    </row>
+    <row r="779">
+      <c r="A779" s="2" t="n">
+        <v>46135</v>
+      </c>
+      <c r="B779" t="inlineStr">
+        <is>
+          <t>龟排腱</t>
+        </is>
+      </c>
+      <c r="C779" t="n">
+        <v>71.59</v>
+      </c>
+      <c r="D779" t="n">
+        <v>71.98</v>
+      </c>
+      <c r="E779" t="n">
+        <v>71.51000000000001</v>
+      </c>
+      <c r="F779" t="n">
+        <v>71.59999999999999</v>
+      </c>
+    </row>
+    <row r="780">
+      <c r="A780" s="2" t="n">
+        <v>46136</v>
+      </c>
+      <c r="B780" t="inlineStr">
+        <is>
+          <t>牛前八件套</t>
+        </is>
+      </c>
+      <c r="C780" t="n">
+        <v>58.18</v>
+      </c>
+      <c r="D780" t="n">
+        <v>58.54</v>
+      </c>
+      <c r="E780" t="n">
+        <v>57.97</v>
+      </c>
+      <c r="F780" t="n">
+        <v>58.4</v>
+      </c>
+    </row>
+    <row r="781">
+      <c r="A781" s="2" t="n">
+        <v>46136</v>
+      </c>
+      <c r="B781" t="inlineStr">
+        <is>
+          <t>龟排腱</t>
+        </is>
+      </c>
+      <c r="C781" t="n">
+        <v>71.34999999999999</v>
+      </c>
+      <c r="D781" t="n">
+        <v>72</v>
+      </c>
+      <c r="E781" t="n">
+        <v>71.12</v>
+      </c>
+      <c r="F781" t="n">
+        <v>71.59999999999999</v>
+      </c>
+    </row>
+    <row r="782">
+      <c r="A782" s="2" t="n">
+        <v>46139</v>
+      </c>
+      <c r="B782" t="inlineStr">
+        <is>
+          <t>牛前八件套</t>
+        </is>
+      </c>
+      <c r="C782" t="n">
+        <v>58.33</v>
+      </c>
+      <c r="D782" t="n">
+        <v>58.58</v>
+      </c>
+      <c r="E782" t="n">
+        <v>58.09</v>
+      </c>
+      <c r="F782" t="n">
+        <v>58.3</v>
+      </c>
+    </row>
+    <row r="783">
+      <c r="A783" s="2" t="n">
+        <v>46139</v>
+      </c>
+      <c r="B783" t="inlineStr">
+        <is>
+          <t>龟排腱</t>
+        </is>
+      </c>
+      <c r="C783" t="n">
+        <v>71.73</v>
+      </c>
+      <c r="D783" t="n">
+        <v>72.15000000000001</v>
+      </c>
+      <c r="E783" t="n">
+        <v>71.53</v>
+      </c>
+      <c r="F783" t="n">
+        <v>71.8</v>
+      </c>
+    </row>
+    <row r="784">
+      <c r="A784" s="2" t="n">
+        <v>46140</v>
+      </c>
+      <c r="B784" t="inlineStr">
+        <is>
+          <t>牛前八件套</t>
+        </is>
+      </c>
+      <c r="C784" t="n">
+        <v>58.2</v>
+      </c>
+      <c r="D784" t="n">
+        <v>58.41</v>
+      </c>
+      <c r="E784" t="n">
+        <v>57.87</v>
+      </c>
+      <c r="F784" t="n">
+        <v>58.2</v>
+      </c>
+    </row>
+    <row r="785">
+      <c r="A785" s="2" t="n">
+        <v>46140</v>
+      </c>
+      <c r="B785" t="inlineStr">
+        <is>
+          <t>龟排腱</t>
+        </is>
+      </c>
+      <c r="C785" t="n">
+        <v>71.90000000000001</v>
+      </c>
+      <c r="D785" t="n">
+        <v>72.09999999999999</v>
+      </c>
+      <c r="E785" t="n">
+        <v>71.8</v>
+      </c>
+      <c r="F785" t="n">
+        <v>71.90000000000001</v>
+      </c>
+    </row>
+    <row r="786">
+      <c r="A786" s="2" t="n">
+        <v>46141</v>
+      </c>
+      <c r="B786" t="inlineStr">
+        <is>
+          <t>牛前八件套</t>
+        </is>
+      </c>
+      <c r="C786" t="n">
+        <v>58.12</v>
+      </c>
+      <c r="D786" t="n">
+        <v>58.35</v>
+      </c>
+      <c r="E786" t="n">
+        <v>57.88</v>
+      </c>
+      <c r="F786" t="n">
+        <v>58.1</v>
+      </c>
+    </row>
+    <row r="787">
+      <c r="A787" s="2" t="n">
+        <v>46141</v>
+      </c>
+      <c r="B787" t="inlineStr">
+        <is>
+          <t>龟排腱</t>
+        </is>
+      </c>
+      <c r="C787" t="n">
+        <v>71.53</v>
+      </c>
+      <c r="D787" t="n">
+        <v>72.42</v>
+      </c>
+      <c r="E787" t="n">
+        <v>71.39</v>
+      </c>
+      <c r="F787" t="n">
+        <v>71.90000000000001</v>
+      </c>
+    </row>
+    <row r="788">
+      <c r="A788" s="2" t="n">
+        <v>46142</v>
+      </c>
+      <c r="B788" t="inlineStr">
+        <is>
+          <t>牛前八件套</t>
+        </is>
+      </c>
+      <c r="C788" t="n">
+        <v>58.13</v>
+      </c>
+      <c r="D788" t="n">
+        <v>58.25</v>
+      </c>
+      <c r="E788" t="n">
+        <v>58.09</v>
+      </c>
+      <c r="F788" t="n">
+        <v>58.1</v>
+      </c>
+    </row>
+    <row r="789">
+      <c r="A789" s="2" t="n">
+        <v>46142</v>
+      </c>
+      <c r="B789" t="inlineStr">
+        <is>
+          <t>龟排腱</t>
+        </is>
+      </c>
+      <c r="C789" t="n">
+        <v>71.95999999999999</v>
+      </c>
+      <c r="D789" t="n">
+        <v>72.34</v>
+      </c>
+      <c r="E789" t="n">
+        <v>71.68000000000001</v>
+      </c>
+      <c r="F789" t="n">
+        <v>72</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>